<commit_message>
DATA. Assess para USA
</commit_message>
<xml_diff>
--- a/data/usa/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
+++ b/data/usa/p6_deployment/data_preparation/clean_data/df_match_player_cleaned.xlsx
@@ -425,118 +425,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:A17"/>
+  <dimension ref="A2:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>hQiNHHd2</t>
+          <t>hIoLKAg0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>C6QBlj7R</t>
+          <t>KEflYcbt</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>dbI3Q902</t>
+          <t>EyfhXHDn</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>zkH7PTF8</t>
+          <t>SvbdWyTh</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>UPVAOmVE</t>
+          <t>AoWGqXpJ</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>8GUEN7pL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>juKJMRaR</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Usy7kWiL</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>lSHwpAFr</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>MNAkH5Nl</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>S0BoIo8r</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>0E9gGPxe</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>Ik4bFqh1</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>dt32E377</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>vqenBDBt</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>SWX9C8ZI</t>
+          <t>trWntSE7</t>
         </is>
       </c>
     </row>

</xml_diff>